<commit_message>
Fix garbled Chinese meaning for in season
英-全民英檢(上) U5 的中文被亂碼污染成「令另的」；修正為「當季的」，
並順手把例句翻譯裡同樣的亂碼文字清乾淨。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/english.xlsx
+++ b/docs/english.xlsx
@@ -32295,13 +32295,13 @@
         <v>ph.</v>
       </c>
       <c r="F175" t="str">
-        <v>令另的</v>
+        <v>當季的</v>
       </c>
       <c r="G175" t="str">
         <v>Strawberries are currently in season and very sweet.</v>
       </c>
       <c r="H175" t="str">
-        <v>草莓目前正值令另的季節，非常甜。</v>
+        <v>草莓目前正值產季，非常甜。</v>
       </c>
     </row>
     <row r="176">

</xml_diff>

<commit_message>
Add GEPT U5 vocab from Win Win English Village U3 listening test
Add 20 words (tag U5) to the 全民英檢-補充1 sheet and regenerate
json/english.json.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/english.xlsx
+++ b/docs/english.xlsx
@@ -50456,7 +50456,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H114"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -52824,10 +52824,530 @@
         <v>我們星期六晚上請了一位保母。</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B95" t="str">
+        <v>put up</v>
+      </c>
+      <c r="C95" t="str">
+        <v>put up</v>
+      </c>
+      <c r="D95" t="str">
+        <v>[pʊt ʌp]</v>
+      </c>
+      <c r="E95" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F95" t="str">
+        <v>張貼</v>
+      </c>
+      <c r="G95" t="str">
+        <v>They put up posters all over the school.</v>
+      </c>
+      <c r="H95" t="str">
+        <v>他們在學校到處張貼海報。</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B96" t="str">
+        <v>poster</v>
+      </c>
+      <c r="C96" t="str">
+        <v>post-er</v>
+      </c>
+      <c r="D96" t="str">
+        <v>['postɚ]</v>
+      </c>
+      <c r="E96" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F96" t="str">
+        <v>海報</v>
+      </c>
+      <c r="G96" t="str">
+        <v>There is a new poster on the wall.</v>
+      </c>
+      <c r="H96" t="str">
+        <v>牆上有一張新海報。</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B97" t="str">
+        <v>make a phone call</v>
+      </c>
+      <c r="C97" t="str">
+        <v>make a phone call</v>
+      </c>
+      <c r="D97" t="str">
+        <v>[mek ə fon kɔl]</v>
+      </c>
+      <c r="E97" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F97" t="str">
+        <v>打電話</v>
+      </c>
+      <c r="G97" t="str">
+        <v>I need to make a phone call to my mom.</v>
+      </c>
+      <c r="H97" t="str">
+        <v>我需要打電話給我媽媽。</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B98" t="str">
+        <v>invitation</v>
+      </c>
+      <c r="C98" t="str">
+        <v>in-vi-ta-tion</v>
+      </c>
+      <c r="D98" t="str">
+        <v>[,ɪnvə'teʃən]</v>
+      </c>
+      <c r="E98" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F98" t="str">
+        <v>邀請函</v>
+      </c>
+      <c r="G98" t="str">
+        <v>She sent an invitation to all her friends.</v>
+      </c>
+      <c r="H98" t="str">
+        <v>她寄了邀請函給所有的朋友。</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B99" t="str">
+        <v>stomach</v>
+      </c>
+      <c r="C99" t="str">
+        <v>stom-ach</v>
+      </c>
+      <c r="D99" t="str">
+        <v>['stʌmək]</v>
+      </c>
+      <c r="E99" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F99" t="str">
+        <v>胃</v>
+      </c>
+      <c r="G99" t="str">
+        <v>My stomach hurts after eating too much.</v>
+      </c>
+      <c r="H99" t="str">
+        <v>我吃太多之後胃很痛。</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B100" t="str">
+        <v>around the corner</v>
+      </c>
+      <c r="C100" t="str">
+        <v>around the corner</v>
+      </c>
+      <c r="D100" t="str">
+        <v>[ə'raʊnd ðə 'kɔrnɚ]</v>
+      </c>
+      <c r="E100" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F100" t="str">
+        <v>轉角</v>
+      </c>
+      <c r="G100" t="str">
+        <v>The bakery is just around the corner.</v>
+      </c>
+      <c r="H100" t="str">
+        <v>那家麵包店就在轉角。</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B101" t="str">
+        <v>lovely</v>
+      </c>
+      <c r="C101" t="str">
+        <v>love-ly</v>
+      </c>
+      <c r="D101" t="str">
+        <v>['lʌvlɪ]</v>
+      </c>
+      <c r="E101" t="str">
+        <v>a.</v>
+      </c>
+      <c r="F101" t="str">
+        <v>美好的/可愛的</v>
+      </c>
+      <c r="G101" t="str">
+        <v>What a lovely garden this is!</v>
+      </c>
+      <c r="H101" t="str">
+        <v>這是一個多麼美好的花園啊！</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B102" t="str">
+        <v>the lead role</v>
+      </c>
+      <c r="C102" t="str">
+        <v>the lead role</v>
+      </c>
+      <c r="D102" t="str">
+        <v>[ðə lid rol]</v>
+      </c>
+      <c r="E102" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F102" t="str">
+        <v>主角</v>
+      </c>
+      <c r="G102" t="str">
+        <v>She played the lead role in the school play.</v>
+      </c>
+      <c r="H102" t="str">
+        <v>她在學校戲劇中飾演主角。</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B103" t="str">
+        <v>opportunity</v>
+      </c>
+      <c r="C103" t="str">
+        <v>op-por-tu-ni-ty</v>
+      </c>
+      <c r="D103" t="str">
+        <v>[,ɑpɚ'tunətɪ]</v>
+      </c>
+      <c r="E103" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F103" t="str">
+        <v>機會</v>
+      </c>
+      <c r="G103" t="str">
+        <v>This is a great opportunity to learn English.</v>
+      </c>
+      <c r="H103" t="str">
+        <v>這是一個學英文的好機會。</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B104" t="str">
+        <v>ancient</v>
+      </c>
+      <c r="C104" t="str">
+        <v>an-cient</v>
+      </c>
+      <c r="D104" t="str">
+        <v>['enʃənt]</v>
+      </c>
+      <c r="E104" t="str">
+        <v>a.</v>
+      </c>
+      <c r="F104" t="str">
+        <v>古代的</v>
+      </c>
+      <c r="G104" t="str">
+        <v>We visited an ancient castle in Europe.</v>
+      </c>
+      <c r="H104" t="str">
+        <v>我們參觀了歐洲的一座古代城堡。</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B105" t="str">
+        <v>dessert</v>
+      </c>
+      <c r="C105" t="str">
+        <v>des-sert</v>
+      </c>
+      <c r="D105" t="str">
+        <v>[dɪ'zɝt]</v>
+      </c>
+      <c r="E105" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F105" t="str">
+        <v>點心</v>
+      </c>
+      <c r="G105" t="str">
+        <v>I always save room for dessert.</v>
+      </c>
+      <c r="H105" t="str">
+        <v>我總是會留肚子吃點心。</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B106" t="str">
+        <v>main course</v>
+      </c>
+      <c r="C106" t="str">
+        <v>main course</v>
+      </c>
+      <c r="D106" t="str">
+        <v>[men kɔrs]</v>
+      </c>
+      <c r="E106" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F106" t="str">
+        <v>主餐</v>
+      </c>
+      <c r="G106" t="str">
+        <v>The main course was steak with vegetables.</v>
+      </c>
+      <c r="H106" t="str">
+        <v>主餐是牛排配蔬菜。</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B107" t="str">
+        <v>suggest</v>
+      </c>
+      <c r="C107" t="str">
+        <v>sug-gest</v>
+      </c>
+      <c r="D107" t="str">
+        <v>[səg'dʒɛst]</v>
+      </c>
+      <c r="E107" t="str">
+        <v>v.</v>
+      </c>
+      <c r="F107" t="str">
+        <v>建議</v>
+      </c>
+      <c r="G107" t="str">
+        <v>I suggest we leave early to avoid traffic.</v>
+      </c>
+      <c r="H107" t="str">
+        <v>我建議我們早點出發以避開塞車。</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B108" t="str">
+        <v>wet</v>
+      </c>
+      <c r="C108" t="str">
+        <v>wet</v>
+      </c>
+      <c r="D108" t="str">
+        <v>[wɛt]</v>
+      </c>
+      <c r="E108" t="str">
+        <v>a.</v>
+      </c>
+      <c r="F108" t="str">
+        <v>溼的</v>
+      </c>
+      <c r="G108" t="str">
+        <v>My shoes got wet in the rain.</v>
+      </c>
+      <c r="H108" t="str">
+        <v>我的鞋子在雨中溼了。</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B109" t="str">
+        <v>weather</v>
+      </c>
+      <c r="C109" t="str">
+        <v>weath-er</v>
+      </c>
+      <c r="D109" t="str">
+        <v>['wɛðɚ]</v>
+      </c>
+      <c r="E109" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F109" t="str">
+        <v>天氣</v>
+      </c>
+      <c r="G109" t="str">
+        <v>The weather is very nice today.</v>
+      </c>
+      <c r="H109" t="str">
+        <v>今天天氣很好。</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B110" t="str">
+        <v>stomachache</v>
+      </c>
+      <c r="C110" t="str">
+        <v>stom-ach-ache</v>
+      </c>
+      <c r="D110" t="str">
+        <v>['stʌməkˌek]</v>
+      </c>
+      <c r="E110" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F110" t="str">
+        <v>胃痛</v>
+      </c>
+      <c r="G110" t="str">
+        <v>He has a stomachache after eating too fast.</v>
+      </c>
+      <c r="H110" t="str">
+        <v>他吃太快之後胃痛。</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B111" t="str">
+        <v>examine</v>
+      </c>
+      <c r="C111" t="str">
+        <v>ex-am-ine</v>
+      </c>
+      <c r="D111" t="str">
+        <v>[ɪg'zæmɪn]</v>
+      </c>
+      <c r="E111" t="str">
+        <v>v.</v>
+      </c>
+      <c r="F111" t="str">
+        <v>檢查</v>
+      </c>
+      <c r="G111" t="str">
+        <v>The doctor will examine your throat.</v>
+      </c>
+      <c r="H111" t="str">
+        <v>醫生將會檢查你的喉嚨。</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B112" t="str">
+        <v>perform</v>
+      </c>
+      <c r="C112" t="str">
+        <v>per-form</v>
+      </c>
+      <c r="D112" t="str">
+        <v>[pɚ'fɔrm]</v>
+      </c>
+      <c r="E112" t="str">
+        <v>v.</v>
+      </c>
+      <c r="F112" t="str">
+        <v>表演/檢測</v>
+      </c>
+      <c r="G112" t="str">
+        <v>The band will perform at the concert tonight.</v>
+      </c>
+      <c r="H112" t="str">
+        <v>這個樂團今晚將在演唱會上表演。</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B113" t="str">
+        <v>boarding pass</v>
+      </c>
+      <c r="C113" t="str">
+        <v>boarding pass</v>
+      </c>
+      <c r="D113" t="str">
+        <v>['bɔrdɪŋ pæs]</v>
+      </c>
+      <c r="E113" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F113" t="str">
+        <v>登機證</v>
+      </c>
+      <c r="G113" t="str">
+        <v>Please show your boarding pass at the gate.</v>
+      </c>
+      <c r="H113" t="str">
+        <v>請在登機門出示你的登機證。</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>U5</v>
+      </c>
+      <c r="B114" t="str">
+        <v>private</v>
+      </c>
+      <c r="C114" t="str">
+        <v>pri-vate</v>
+      </c>
+      <c r="D114" t="str">
+        <v>['praɪvɪt]</v>
+      </c>
+      <c r="E114" t="str">
+        <v>a.</v>
+      </c>
+      <c r="F114" t="str">
+        <v>私人的</v>
+      </c>
+      <c r="G114" t="str">
+        <v>This is a private conversation.</v>
+      </c>
+      <c r="H114" t="str">
+        <v>這是一段私人的對話。</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H114"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add GEPT U6 vocab from Win Win English Village U3 reading test
Add 20 words (tag U6) to the 全民英檢-補充1 sheet and regenerate
json/english.json.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/english.xlsx
+++ b/docs/english.xlsx
@@ -50456,7 +50456,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H134"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -53344,10 +53344,530 @@
         <v>這是一段私人的對話。</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B115" t="str">
+        <v>celebrate</v>
+      </c>
+      <c r="C115" t="str">
+        <v>ce-le-brate</v>
+      </c>
+      <c r="D115" t="str">
+        <v>['sɛlə,bret]</v>
+      </c>
+      <c r="E115" t="str">
+        <v>v.</v>
+      </c>
+      <c r="F115" t="str">
+        <v>慶祝</v>
+      </c>
+      <c r="G115" t="str">
+        <v>We celebrate Christmas with our family.</v>
+      </c>
+      <c r="H115" t="str">
+        <v>我們和家人一起慶祝聖誕節。</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B116" t="str">
+        <v>figure</v>
+      </c>
+      <c r="C116" t="str">
+        <v>fi-gure</v>
+      </c>
+      <c r="D116" t="str">
+        <v>['fɪgjɚ]</v>
+      </c>
+      <c r="E116" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F116" t="str">
+        <v>角色</v>
+      </c>
+      <c r="G116" t="str">
+        <v>Batman is a famous figure in comic books.</v>
+      </c>
+      <c r="H116" t="str">
+        <v>蝙蝠俠是漫畫裡很有名的角色。</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B117" t="str">
+        <v>traditionally</v>
+      </c>
+      <c r="C117" t="str">
+        <v>tra-di-tion-al-ly</v>
+      </c>
+      <c r="D117" t="str">
+        <v>[trə'dɪʃənlɪ]</v>
+      </c>
+      <c r="E117" t="str">
+        <v>adv.</v>
+      </c>
+      <c r="F117" t="str">
+        <v>傳統地</v>
+      </c>
+      <c r="G117" t="str">
+        <v>Traditionally, people eat moon cakes at the Moon Festival.</v>
+      </c>
+      <c r="H117" t="str">
+        <v>傳統上，人們在中秋節吃月餅。</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B118" t="str">
+        <v>greeting card</v>
+      </c>
+      <c r="C118" t="str">
+        <v>greeting card</v>
+      </c>
+      <c r="D118" t="str">
+        <v>['gritɪŋ kɑrd]</v>
+      </c>
+      <c r="E118" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F118" t="str">
+        <v>賀卡</v>
+      </c>
+      <c r="G118" t="str">
+        <v>I made a greeting card for my teacher.</v>
+      </c>
+      <c r="H118" t="str">
+        <v>我做了一張賀卡給老師。</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Ger-ma-ny</v>
+      </c>
+      <c r="D119" t="str">
+        <v>['dʒɝmənɪ]</v>
+      </c>
+      <c r="E119" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F119" t="str">
+        <v>德國</v>
+      </c>
+      <c r="G119" t="str">
+        <v>My uncle lives in Germany.</v>
+      </c>
+      <c r="H119" t="str">
+        <v>我叔叔住在德國。</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B120" t="str">
+        <v>toward</v>
+      </c>
+      <c r="C120" t="str">
+        <v>to-ward</v>
+      </c>
+      <c r="D120" t="str">
+        <v>[tə'wɔrd]</v>
+      </c>
+      <c r="E120" t="str">
+        <v>prep.</v>
+      </c>
+      <c r="F120" t="str">
+        <v>朝向</v>
+      </c>
+      <c r="G120" t="str">
+        <v>The dog ran toward me.</v>
+      </c>
+      <c r="H120" t="str">
+        <v>那隻狗朝我跑過來。</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B121" t="str">
+        <v>during</v>
+      </c>
+      <c r="C121" t="str">
+        <v>du-ring</v>
+      </c>
+      <c r="D121" t="str">
+        <v>['djʊrɪŋ]</v>
+      </c>
+      <c r="E121" t="str">
+        <v>prep.</v>
+      </c>
+      <c r="F121" t="str">
+        <v>在…期間</v>
+      </c>
+      <c r="G121" t="str">
+        <v>Please don't talk during the test.</v>
+      </c>
+      <c r="H121" t="str">
+        <v>考試期間請不要講話。</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B122" t="str">
+        <v>against</v>
+      </c>
+      <c r="C122" t="str">
+        <v>a-gainst</v>
+      </c>
+      <c r="D122" t="str">
+        <v>[ə'gɛnst]</v>
+      </c>
+      <c r="E122" t="str">
+        <v>prep.</v>
+      </c>
+      <c r="F122" t="str">
+        <v>反對</v>
+      </c>
+      <c r="G122" t="str">
+        <v>Many people are against the new rule.</v>
+      </c>
+      <c r="H122" t="str">
+        <v>很多人反對這條新規定。</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B123" t="str">
+        <v>including</v>
+      </c>
+      <c r="C123" t="str">
+        <v>in-clu-ding</v>
+      </c>
+      <c r="D123" t="str">
+        <v>[ɪn'kludɪŋ]</v>
+      </c>
+      <c r="E123" t="str">
+        <v>prep.</v>
+      </c>
+      <c r="F123" t="str">
+        <v>包括</v>
+      </c>
+      <c r="G123" t="str">
+        <v>Ten students, including me, joined the club.</v>
+      </c>
+      <c r="H123" t="str">
+        <v>包括我在內，有十個學生加入了社團。</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B124" t="str">
+        <v>contain</v>
+      </c>
+      <c r="C124" t="str">
+        <v>con-tain</v>
+      </c>
+      <c r="D124" t="str">
+        <v>[kən'ten]</v>
+      </c>
+      <c r="E124" t="str">
+        <v>v.</v>
+      </c>
+      <c r="F124" t="str">
+        <v>含有</v>
+      </c>
+      <c r="G124" t="str">
+        <v>This drink contains a lot of sugar.</v>
+      </c>
+      <c r="H124" t="str">
+        <v>這杯飲料含有很多糖。</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B125" t="str">
+        <v>damage</v>
+      </c>
+      <c r="C125" t="str">
+        <v>da-mage</v>
+      </c>
+      <c r="D125" t="str">
+        <v>['dæmɪdʒ]</v>
+      </c>
+      <c r="E125" t="str">
+        <v>v.</v>
+      </c>
+      <c r="F125" t="str">
+        <v>傷害</v>
+      </c>
+      <c r="G125" t="str">
+        <v>Too much sun can damage your skin.</v>
+      </c>
+      <c r="H125" t="str">
+        <v>太多陽光會傷害你的皮膚。</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B126" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="C126" t="str">
+        <v>pa-ssen-ger</v>
+      </c>
+      <c r="D126" t="str">
+        <v>['pæsəndʒɚ]</v>
+      </c>
+      <c r="E126" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F126" t="str">
+        <v>乘客</v>
+      </c>
+      <c r="G126" t="str">
+        <v>There are fifty passengers on the bus.</v>
+      </c>
+      <c r="H126" t="str">
+        <v>公車上有五十位乘客。</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B127" t="str">
+        <v>height</v>
+      </c>
+      <c r="C127" t="str">
+        <v>height</v>
+      </c>
+      <c r="D127" t="str">
+        <v>[haɪt]</v>
+      </c>
+      <c r="E127" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F127" t="str">
+        <v>高度</v>
+      </c>
+      <c r="G127" t="str">
+        <v>What is the height of that building?</v>
+      </c>
+      <c r="H127" t="str">
+        <v>那棟大樓的高度是多少？</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B128" t="str">
+        <v>delay</v>
+      </c>
+      <c r="C128" t="str">
+        <v>de-lay</v>
+      </c>
+      <c r="D128" t="str">
+        <v>[dɪ'le]</v>
+      </c>
+      <c r="E128" t="str">
+        <v>v.</v>
+      </c>
+      <c r="F128" t="str">
+        <v>延遲</v>
+      </c>
+      <c r="G128" t="str">
+        <v>The bad weather delayed our flight.</v>
+      </c>
+      <c r="H128" t="str">
+        <v>壞天氣延遲了我們的班機。</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B129" t="str">
+        <v>energy</v>
+      </c>
+      <c r="C129" t="str">
+        <v>e-ner-gy</v>
+      </c>
+      <c r="D129" t="str">
+        <v>['ɛnɚdʒɪ]</v>
+      </c>
+      <c r="E129" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F129" t="str">
+        <v>能源</v>
+      </c>
+      <c r="G129" t="str">
+        <v>We should save energy at home.</v>
+      </c>
+      <c r="H129" t="str">
+        <v>我們在家應該節約能源。</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B130" t="str">
+        <v>environment</v>
+      </c>
+      <c r="C130" t="str">
+        <v>en-vi-ron-ment</v>
+      </c>
+      <c r="D130" t="str">
+        <v>[ɪn'vaɪrənmənt]</v>
+      </c>
+      <c r="E130" t="str">
+        <v>n.</v>
+      </c>
+      <c r="F130" t="str">
+        <v>環境</v>
+      </c>
+      <c r="G130" t="str">
+        <v>We must protect the environment.</v>
+      </c>
+      <c r="H130" t="str">
+        <v>我們必須保護環境。</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B131" t="str">
+        <v>find fault with</v>
+      </c>
+      <c r="C131" t="str">
+        <v>find fault with</v>
+      </c>
+      <c r="D131" t="str">
+        <v>[faɪnd fɔlt wɪð]</v>
+      </c>
+      <c r="E131" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F131" t="str">
+        <v>挑剔…錯誤</v>
+      </c>
+      <c r="G131" t="str">
+        <v>My sister always finds fault with my cooking.</v>
+      </c>
+      <c r="H131" t="str">
+        <v>我姊姊總是挑剔我煮的菜。</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B132" t="str">
+        <v>be crazy about</v>
+      </c>
+      <c r="C132" t="str">
+        <v>be crazy about</v>
+      </c>
+      <c r="D132" t="str">
+        <v>[bi 'krezɪ ə'baʊt]</v>
+      </c>
+      <c r="E132" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F132" t="str">
+        <v>瘋迷於…</v>
+      </c>
+      <c r="G132" t="str">
+        <v>Tom is crazy about basketball.</v>
+      </c>
+      <c r="H132" t="str">
+        <v>湯姆瘋迷於籃球。</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B133" t="str">
+        <v>come up with</v>
+      </c>
+      <c r="C133" t="str">
+        <v>come up with</v>
+      </c>
+      <c r="D133" t="str">
+        <v>[kʌm ʌp wɪð]</v>
+      </c>
+      <c r="E133" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F133" t="str">
+        <v>想出(辦法)</v>
+      </c>
+      <c r="G133" t="str">
+        <v>She came up with a great idea.</v>
+      </c>
+      <c r="H133" t="str">
+        <v>她想出了一個很棒的點子。</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>U6</v>
+      </c>
+      <c r="B134" t="str">
+        <v>come into contact with</v>
+      </c>
+      <c r="C134" t="str">
+        <v>come into contact with</v>
+      </c>
+      <c r="D134" t="str">
+        <v>[kʌm 'ɪntu 'kɑntækt wɪð]</v>
+      </c>
+      <c r="E134" t="str">
+        <v>ph.</v>
+      </c>
+      <c r="F134" t="str">
+        <v>接觸/碰到</v>
+      </c>
+      <c r="G134" t="str">
+        <v>Wash your hands if you come into contact with the paint.</v>
+      </c>
+      <c r="H134" t="str">
+        <v>如果你碰到油漆，要洗手喔。</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H114"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H134"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>